<commit_message>
modeling and documentation mostly done, I believe
</commit_message>
<xml_diff>
--- a/predicciones_mar5_13_2026.xlsx
+++ b/predicciones_mar5_13_2026.xlsx
@@ -16,20 +16,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,22 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,87 +417,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>modelo_1</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
-          <t>Pronóstico</t>
+          <t>modelo_2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46084</v>
+      <c r="A2" t="n">
+        <v>17.6397887855245</v>
       </c>
       <c r="B2" t="n">
-        <v>17.35297777028803</v>
+        <v>17.51753257649803</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>46085</v>
+      <c r="A3" t="n">
+        <v>17.6033861474459</v>
       </c>
       <c r="B3" t="n">
-        <v>17.35514364409503</v>
+        <v>17.50739154101716</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46086</v>
+      <c r="A4" t="n">
+        <v>17.73262584594179</v>
       </c>
       <c r="B4" t="n">
-        <v>17.35786654287827</v>
+        <v>17.48798704126905</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46087</v>
+      <c r="A5" t="n">
+        <v>18.10692848415912</v>
       </c>
       <c r="B5" t="n">
-        <v>17.35949955569166</v>
+        <v>17.47572031836453</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>46088</v>
+      <c r="A6" t="n">
+        <v>17.92862865948543</v>
       </c>
       <c r="B6" t="n">
-        <v>17.36061672661468</v>
+        <v>17.44651128494709</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>46089</v>
+      <c r="A7" t="n">
+        <v>18.02391745666148</v>
       </c>
       <c r="B7" t="n">
-        <v>17.36021903785456</v>
+        <v>17.44145935356578</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46090</v>
+      <c r="A8" t="n">
+        <v>17.9875148193572</v>
       </c>
       <c r="B8" t="n">
-        <v>17.36330833909048</v>
+        <v>17.43649325083044</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>46091</v>
+      <c r="A9" t="n">
+        <v>18.11675451790454</v>
       </c>
       <c r="B9" t="n">
-        <v>17.36595226935895</v>
+        <v>17.42546353877913</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46092</v>
+      <c r="A10" t="n">
+        <v>18.49105715612529</v>
       </c>
       <c r="B10" t="n">
-        <v>17.36757194232065</v>
+        <v>17.42987783999636</v>
       </c>
     </row>
   </sheetData>

</xml_diff>